<commit_message>
fix: actualizacion del excel
</commit_message>
<xml_diff>
--- a/excels/Horarios ICIF 202620 Enviado 3.xlsx
+++ b/excels/Horarios ICIF 202620 Enviado 3.xlsx
@@ -8,25 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BACAEA7D-EA86-4CE2-996D-D38C835E4736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BEAAEF1-C37C-4B47-BCCF-3F4F84225683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Semestre 2" sheetId="5" r:id="rId1"/>
-    <sheet name="Semestre 3" sheetId="4" r:id="rId2"/>
-    <sheet name="Semestre 4" sheetId="2" r:id="rId3"/>
-    <sheet name="Semestre 6_nueva" sheetId="6" r:id="rId4"/>
-    <sheet name="Semestre 6_antigua" sheetId="7" r:id="rId5"/>
-    <sheet name="Semestre 8" sheetId="3" r:id="rId6"/>
-    <sheet name="Semestre 10" sheetId="8" r:id="rId7"/>
+    <sheet name="Semestre 1" sheetId="9" r:id="rId1"/>
+    <sheet name="Semestre 2" sheetId="5" r:id="rId2"/>
+    <sheet name="Semestre 3" sheetId="4" r:id="rId3"/>
+    <sheet name="Semestre 4" sheetId="2" r:id="rId4"/>
+    <sheet name="Semestre 6_nueva" sheetId="6" r:id="rId5"/>
+    <sheet name="Semestre 6_antigua" sheetId="7" r:id="rId6"/>
+    <sheet name="Semestre 8" sheetId="3" r:id="rId7"/>
+    <sheet name="Semestre 10" sheetId="8" r:id="rId8"/>
+    <sheet name="Ingleses" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2692" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3154" uniqueCount="368">
   <si>
     <t>NRC</t>
   </si>
@@ -1037,6 +1039,99 @@
   </si>
   <si>
     <t>13914</t>
+  </si>
+  <si>
+    <t>12073</t>
+  </si>
+  <si>
+    <t>0010</t>
+  </si>
+  <si>
+    <t>ALGEBRA</t>
+  </si>
+  <si>
+    <t>ICOM</t>
+  </si>
+  <si>
+    <t>12077</t>
+  </si>
+  <si>
+    <t>4282</t>
+  </si>
+  <si>
+    <t>0007</t>
+  </si>
+  <si>
+    <t>4284</t>
+  </si>
+  <si>
+    <t>5368</t>
+  </si>
+  <si>
+    <t>8442</t>
+  </si>
+  <si>
+    <t>0008</t>
+  </si>
+  <si>
+    <t>INTRODUCCION AL CALCULO</t>
+  </si>
+  <si>
+    <t>REYES/MONSALVE</t>
+  </si>
+  <si>
+    <t>ICMI</t>
+  </si>
+  <si>
+    <t>8443</t>
+  </si>
+  <si>
+    <t>ICIV</t>
+  </si>
+  <si>
+    <t>4281</t>
+  </si>
+  <si>
+    <t>5366</t>
+  </si>
+  <si>
+    <t>5367</t>
+  </si>
+  <si>
+    <t>8441</t>
+  </si>
+  <si>
+    <t>5777</t>
+  </si>
+  <si>
+    <t>1416</t>
+  </si>
+  <si>
+    <t>INGLES II</t>
+  </si>
+  <si>
+    <t>MARIA</t>
+  </si>
+  <si>
+    <t>ESCOBAR/AGURTO</t>
+  </si>
+  <si>
+    <t>5875</t>
+  </si>
+  <si>
+    <t>1431</t>
+  </si>
+  <si>
+    <t>INGLES TECNICO</t>
+  </si>
+  <si>
+    <t>5876</t>
+  </si>
+  <si>
+    <t>FELIPE</t>
+  </si>
+  <si>
+    <t>BENAVENTE/ULLOA</t>
   </si>
 </sst>
 </file>
@@ -1464,6 +1559,1318 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33AB8C9A-831E-4FA0-B6F6-A0D2666A1987}">
+  <dimension ref="A1:S27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="7" max="7" width="24.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19">
+      <c r="A2" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="S2" s="2"/>
+    </row>
+    <row r="3" spans="1:19">
+      <c r="A3" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K3" s="2"/>
+      <c r="L3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
+      <c r="A4" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="S4" s="2"/>
+    </row>
+    <row r="5" spans="1:19">
+      <c r="A5" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="K5" s="2"/>
+      <c r="L5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="S5" s="2"/>
+    </row>
+    <row r="6" spans="1:19">
+      <c r="A6" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="S6" s="2"/>
+    </row>
+    <row r="7" spans="1:19">
+      <c r="A7" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L7" s="3"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="S7" s="2"/>
+    </row>
+    <row r="8" spans="1:19">
+      <c r="A8" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K8" s="2"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="R8" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="S8" s="2"/>
+    </row>
+    <row r="9" spans="1:19">
+      <c r="A9" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K9" s="2"/>
+      <c r="L9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="S9" s="2"/>
+    </row>
+    <row r="10" spans="1:19">
+      <c r="A10" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="R10" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="S10" s="2"/>
+    </row>
+    <row r="11" spans="1:19">
+      <c r="A11" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K11" s="2"/>
+      <c r="L11" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="S11" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19">
+      <c r="A12" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K12" s="2"/>
+      <c r="L12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="S12" s="2"/>
+    </row>
+    <row r="13" spans="1:19">
+      <c r="A13" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K13" s="2"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="S13" s="2" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19">
+      <c r="A14" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19">
+      <c r="A15" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K15" s="2"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19">
+      <c r="A16" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="S16" s="1"/>
+    </row>
+    <row r="17" spans="1:19">
+      <c r="A17" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R17" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="S17" s="1"/>
+    </row>
+    <row r="18" spans="1:19">
+      <c r="A18" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+      <c r="Q18" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R18" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="S18" s="1"/>
+    </row>
+    <row r="19" spans="1:19">
+      <c r="A19" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1"/>
+      <c r="Q19" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="R19" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="S19" s="1"/>
+    </row>
+    <row r="20" spans="1:19">
+      <c r="A20" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+      <c r="Q20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="R20" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="S20" s="1" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19">
+      <c r="A21" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="R21" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="S21" s="1"/>
+    </row>
+    <row r="22" spans="1:19">
+      <c r="A22" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R22" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="S22" s="1" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19">
+      <c r="A23" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R23" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="S23" s="1" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19">
+      <c r="A24" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R24" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="S24" s="1" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19">
+      <c r="A25" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R25" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="S25" s="1"/>
+    </row>
+    <row r="26" spans="1:19">
+      <c r="A26" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R26" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="S26" s="1"/>
+    </row>
+    <row r="27" spans="1:19">
+      <c r="A27" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R27" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="S27" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B04450B-4D3A-444A-8C70-833821F0E18C}">
   <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
@@ -3045,7 +4452,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{742B1EB3-54E8-42B1-96A5-AD861CB086AD}">
   <dimension ref="A1:S31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
@@ -4526,7 +5933,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F31639A8-B77F-40D3-A3E2-D8298BF83C8B}">
   <dimension ref="A1:S30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
@@ -5965,7 +7372,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36BD2444-5417-4C3B-ACAC-17D64029070C}">
   <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
@@ -7453,7 +8860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8ABF100-BEC0-4DD6-AD50-C4B8A3F777CB}">
   <dimension ref="A1:S47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
@@ -9576,7 +10983,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BE4429E-CA1B-4529-94AE-CE97ED6F115A}">
   <dimension ref="A1:S29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
@@ -10937,7 +12344,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{939E82A5-8A64-4B2B-8701-1D6FF57E175E}">
   <dimension ref="A1:S17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
@@ -11723,4 +13130,384 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8554B521-5B20-4750-BD74-44BFF8934136}">
+  <dimension ref="A1:T8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="7" max="7" width="14.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20">
+      <c r="A2" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+    </row>
+    <row r="5" spans="1:20">
+      <c r="A5" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+    </row>
+    <row r="6" spans="1:20">
+      <c r="A6" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+    </row>
+    <row r="7" spans="1:20">
+      <c r="A7" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="R7" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+    </row>
+    <row r="8" spans="1:20">
+      <c r="A8" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="S8" s="6"/>
+      <c r="T8" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: correccion en los horarios del excel
</commit_message>
<xml_diff>
--- a/excels/Horarios ICIF 202620 Enviado 3.xlsx
+++ b/excels/Horarios ICIF 202620 Enviado 3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BEAAEF1-C37C-4B47-BCCF-3F4F84225683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B12831-7E1D-42CE-B302-B5809EF04DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Semestre 1" sheetId="9" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3154" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3294" uniqueCount="370">
   <si>
     <t>NRC</t>
   </si>
@@ -1132,6 +1132,12 @@
   </si>
   <si>
     <t>BENAVENTE/ULLOA</t>
+  </si>
+  <si>
+    <t>21668</t>
+  </si>
+  <si>
+    <t>21670</t>
   </si>
 </sst>
 </file>
@@ -7374,7 +7380,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36BD2444-5417-4C3B-ACAC-17D64029070C}">
-  <dimension ref="A1:S33"/>
+  <dimension ref="A1:S45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="7" max="7" width="32.33203125" bestFit="1" customWidth="1"/>
@@ -8449,411 +8455,943 @@
       <c r="S24" s="1"/>
     </row>
     <row r="25" spans="1:19">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="6"/>
+      <c r="P25" s="6"/>
+      <c r="Q25" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="R25" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="S25" s="6"/>
+    </row>
+    <row r="26" spans="1:19">
+      <c r="A26" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="K26" s="6"/>
+      <c r="L26" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="6"/>
+      <c r="P26" s="6"/>
+      <c r="Q26" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="R26" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="S26" s="6"/>
+    </row>
+    <row r="27" spans="1:19">
+      <c r="A27" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L27" s="6"/>
+      <c r="M27" s="6"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
+      <c r="Q27" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="R27" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="S27" s="6"/>
+    </row>
+    <row r="28" spans="1:19">
+      <c r="A28" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="K28" s="6"/>
+      <c r="L28" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M28" s="6"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="R28" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="S28" s="6"/>
+    </row>
+    <row r="29" spans="1:19">
+      <c r="A29" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C25" s="1" t="s">
+      <c r="B29" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D29" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E29" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="G29" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1" t="s">
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K25" s="1" t="s">
+      <c r="K29" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
-      <c r="Q25" s="1" t="s">
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="R25" s="1" t="s">
+      <c r="R29" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="S25" s="1"/>
-    </row>
-    <row r="26" spans="1:19">
-      <c r="A26" s="1" t="s">
+      <c r="S29" s="1"/>
+    </row>
+    <row r="30" spans="1:19">
+      <c r="A30" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="B30" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D30" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E30" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F30" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1" t="s">
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="K30" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L26" s="1"/>
-      <c r="M26" s="1"/>
-      <c r="N26" s="1"/>
-      <c r="O26" s="1"/>
-      <c r="P26" s="1"/>
-      <c r="Q26" s="1" t="s">
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="R26" s="1" t="s">
+      <c r="R30" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="S26" s="1"/>
-    </row>
-    <row r="27" spans="1:19">
-      <c r="A27" s="1" t="s">
+      <c r="S30" s="1"/>
+    </row>
+    <row r="31" spans="1:19">
+      <c r="A31" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C27" s="1" t="s">
+      <c r="B31" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="I27" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J27" s="1" t="s">
+      <c r="J31" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K27" s="1"/>
-      <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
-      <c r="O27" s="1" t="s">
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="P27" s="1"/>
-      <c r="Q27" s="1" t="s">
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="R27" s="1" t="s">
+      <c r="R31" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="S27" s="1"/>
-    </row>
-    <row r="28" spans="1:19">
-      <c r="A28" s="1" t="s">
+      <c r="S31" s="1"/>
+    </row>
+    <row r="32" spans="1:19">
+      <c r="A32" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C28" s="1" t="s">
+      <c r="B32" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F32" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="G32" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="H28" s="1" t="s">
+      <c r="H32" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="I28" s="1" t="s">
+      <c r="I32" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J28" s="1" t="s">
+      <c r="J32" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K28" s="1"/>
-      <c r="L28" s="1"/>
-      <c r="M28" s="1"/>
-      <c r="N28" s="1" t="s">
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O28" s="1"/>
-      <c r="P28" s="1"/>
-      <c r="Q28" s="1" t="s">
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="R28" s="1" t="s">
+      <c r="R32" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="S28" s="1"/>
-    </row>
-    <row r="29" spans="1:19">
-      <c r="A29" s="6" t="s">
+      <c r="S32" s="1"/>
+    </row>
+    <row r="33" spans="1:19">
+      <c r="A33" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="B29" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="C29" s="6" t="s">
+      <c r="B33" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D33" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E33" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F33" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G29" s="6" t="s">
+      <c r="G33" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="H29" s="6" t="s">
+      <c r="H33" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I29" s="6" t="s">
+      <c r="I33" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="J29" s="6" t="s">
+      <c r="J33" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="K29" s="6"/>
-      <c r="L29" s="6" t="s">
+      <c r="K33" s="6"/>
+      <c r="L33" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="M29" s="6"/>
-      <c r="N29" s="6"/>
-      <c r="O29" s="6"/>
-      <c r="P29" s="6"/>
-      <c r="Q29" s="6" t="s">
+      <c r="M33" s="6"/>
+      <c r="N33" s="6"/>
+      <c r="O33" s="6"/>
+      <c r="P33" s="6"/>
+      <c r="Q33" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="R29" s="6" t="s">
+      <c r="R33" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="S29" s="6"/>
-    </row>
-    <row r="30" spans="1:19">
-      <c r="A30" s="6" t="s">
+      <c r="S33" s="6"/>
+    </row>
+    <row r="34" spans="1:19">
+      <c r="A34" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="B30" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="C30" s="6" t="s">
+      <c r="B34" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C34" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D34" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E34" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="F34" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G30" s="6" t="s">
+      <c r="G34" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="H30" s="6" t="s">
+      <c r="H34" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I30" s="6" t="s">
+      <c r="I34" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="J30" s="6" t="s">
+      <c r="J34" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="K30" s="6" t="s">
+      <c r="K34" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="L30" s="6"/>
-      <c r="M30" s="6"/>
-      <c r="N30" s="6"/>
-      <c r="O30" s="6"/>
-      <c r="P30" s="6"/>
-      <c r="Q30" s="6" t="s">
+      <c r="L34" s="6"/>
+      <c r="M34" s="6"/>
+      <c r="N34" s="6"/>
+      <c r="O34" s="6"/>
+      <c r="P34" s="6"/>
+      <c r="Q34" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="R30" s="6" t="s">
+      <c r="R34" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="S30" s="6"/>
-    </row>
-    <row r="31" spans="1:19">
-      <c r="A31" s="6" t="s">
+      <c r="S34" s="6"/>
+    </row>
+    <row r="35" spans="1:19">
+      <c r="A35" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="C31" s="6" t="s">
+      <c r="B35" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C35" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D35" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E35" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="F35" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G31" s="6" t="s">
+      <c r="G35" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="H31" s="6" t="s">
+      <c r="H35" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I31" s="6" t="s">
+      <c r="I35" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="J31" s="6" t="s">
+      <c r="J35" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6" t="s">
+      <c r="K35" s="6"/>
+      <c r="L35" s="6"/>
+      <c r="M35" s="6"/>
+      <c r="N35" s="6"/>
+      <c r="O35" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="P31" s="6"/>
-      <c r="Q31" s="6" t="s">
+      <c r="P35" s="6"/>
+      <c r="Q35" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="R31" s="6" t="s">
+      <c r="R35" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="S31" s="6"/>
-    </row>
-    <row r="32" spans="1:19">
-      <c r="A32" s="6" t="s">
+      <c r="S35" s="6"/>
+    </row>
+    <row r="36" spans="1:19">
+      <c r="A36" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="B32" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="C32" s="6" t="s">
+      <c r="B36" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D36" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E36" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="F36" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="G36" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="H32" s="6" t="s">
+      <c r="H36" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I32" s="6" t="s">
+      <c r="I36" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="J32" s="6" t="s">
+      <c r="J36" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="K32" s="6" t="s">
+      <c r="K36" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="L32" s="6"/>
-      <c r="M32" s="6"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="6"/>
-      <c r="P32" s="6"/>
-      <c r="Q32" s="6" t="s">
+      <c r="L36" s="6"/>
+      <c r="M36" s="6"/>
+      <c r="N36" s="6"/>
+      <c r="O36" s="6"/>
+      <c r="P36" s="6"/>
+      <c r="Q36" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="R32" s="6" t="s">
+      <c r="R36" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="S32" s="6"/>
-    </row>
-    <row r="33" spans="1:19">
-      <c r="A33" s="4" t="s">
+      <c r="S36" s="6"/>
+    </row>
+    <row r="37" spans="1:19">
+      <c r="A37" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="C33" s="4" t="s">
+      <c r="B37" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D37" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E37" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F37" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="G33" s="4" t="s">
+      <c r="G37" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4"/>
-      <c r="O33" s="4"/>
-      <c r="P33" s="4"/>
-      <c r="Q33" s="4" t="s">
+      <c r="H37" s="4"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4"/>
+      <c r="O37" s="4"/>
+      <c r="P37" s="4"/>
+      <c r="Q37" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="R33" s="4" t="s">
+      <c r="R37" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="S33" s="4"/>
+      <c r="S37" s="4"/>
+    </row>
+    <row r="38" spans="1:19">
+      <c r="A38" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K38" s="2"/>
+      <c r="L38" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M38" s="3"/>
+      <c r="N38" s="2"/>
+      <c r="O38" s="2"/>
+      <c r="P38" s="2"/>
+      <c r="Q38" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="R38" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="S38" s="3"/>
+    </row>
+    <row r="39" spans="1:19">
+      <c r="A39" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="K39" s="2"/>
+      <c r="L39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M39" s="3"/>
+      <c r="N39" s="2"/>
+      <c r="O39" s="2"/>
+      <c r="P39" s="2"/>
+      <c r="Q39" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="R39" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="S39" s="3"/>
+    </row>
+    <row r="40" spans="1:19">
+      <c r="A40" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K40" s="2"/>
+      <c r="L40" s="2"/>
+      <c r="M40" s="3"/>
+      <c r="N40" s="2"/>
+      <c r="O40" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="P40" s="2"/>
+      <c r="Q40" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="R40" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="S40" s="3"/>
+    </row>
+    <row r="41" spans="1:19">
+      <c r="A41" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K41" s="2"/>
+      <c r="L41" s="2"/>
+      <c r="M41" s="3"/>
+      <c r="N41" s="2"/>
+      <c r="O41" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="P41" s="2"/>
+      <c r="Q41" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="R41" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="S41" s="3"/>
+    </row>
+    <row r="42" spans="1:19">
+      <c r="A42" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K42" s="2"/>
+      <c r="L42" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M42" s="3"/>
+      <c r="N42" s="2"/>
+      <c r="O42" s="2"/>
+      <c r="P42" s="2"/>
+      <c r="Q42" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="R42" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="S42" s="3"/>
+    </row>
+    <row r="43" spans="1:19">
+      <c r="A43" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="K43" s="2"/>
+      <c r="L43" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M43" s="3"/>
+      <c r="N43" s="2"/>
+      <c r="O43" s="2"/>
+      <c r="P43" s="2"/>
+      <c r="Q43" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="R43" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="S43" s="3"/>
+    </row>
+    <row r="44" spans="1:19">
+      <c r="A44" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="3"/>
+      <c r="N44" s="2"/>
+      <c r="O44" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="P44" s="2"/>
+      <c r="Q44" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="R44" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="S44" s="3"/>
+    </row>
+    <row r="45" spans="1:19">
+      <c r="A45" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K45" s="2"/>
+      <c r="L45" s="2"/>
+      <c r="M45" s="3"/>
+      <c r="N45" s="2"/>
+      <c r="O45" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="P45" s="2"/>
+      <c r="Q45" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="R45" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="S45" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: actualizacion de excel
</commit_message>
<xml_diff>
--- a/excels/Horarios ICIF 202620 Enviado 3.xlsx
+++ b/excels/Horarios ICIF 202620 Enviado 3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B12831-7E1D-42CE-B302-B5809EF04DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC25341-B320-4B88-AF48-6FE23D4CDCE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Semestre 1" sheetId="9" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3294" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3398" uniqueCount="377">
   <si>
     <t>NRC</t>
   </si>
@@ -1138,6 +1138,27 @@
   </si>
   <si>
     <t>21670</t>
+  </si>
+  <si>
+    <t>13757</t>
+  </si>
+  <si>
+    <t>13758</t>
+  </si>
+  <si>
+    <t>T1G</t>
+  </si>
+  <si>
+    <t>13759</t>
+  </si>
+  <si>
+    <t>T1H</t>
+  </si>
+  <si>
+    <t>13760</t>
+  </si>
+  <si>
+    <t>T1I</t>
   </si>
 </sst>
 </file>
@@ -2878,7 +2899,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B04450B-4D3A-444A-8C70-833821F0E18C}">
-  <dimension ref="A1:S33"/>
+  <dimension ref="A1:S41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="6" max="6" width="12.44140625" bestFit="1" customWidth="1"/>
@@ -4452,6 +4473,382 @@
         <v>86</v>
       </c>
       <c r="S33" s="1"/>
+    </row>
+    <row r="34" spans="1:19">
+      <c r="A34" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O34" s="2"/>
+      <c r="P34" s="2"/>
+      <c r="Q34" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="R34" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S34" s="2"/>
+    </row>
+    <row r="35" spans="1:19">
+      <c r="A35" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
+      <c r="O35" s="2"/>
+      <c r="P35" s="2"/>
+      <c r="Q35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="R35" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S35" s="2"/>
+    </row>
+    <row r="36" spans="1:19">
+      <c r="A36" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O36" s="2"/>
+      <c r="P36" s="2"/>
+      <c r="Q36" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="R36" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="S36" s="2"/>
+    </row>
+    <row r="37" spans="1:19">
+      <c r="A37" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K37" s="2"/>
+      <c r="L37" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
+      <c r="P37" s="2"/>
+      <c r="Q37" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="R37" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="S37" s="2"/>
+    </row>
+    <row r="38" spans="1:19">
+      <c r="A38" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K38" s="2"/>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
+      <c r="N38" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O38" s="2"/>
+      <c r="P38" s="2"/>
+      <c r="Q38" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="R38" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="S38" s="2"/>
+    </row>
+    <row r="39" spans="1:19">
+      <c r="A39" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K39" s="2"/>
+      <c r="L39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M39" s="2"/>
+      <c r="N39" s="2"/>
+      <c r="O39" s="2"/>
+      <c r="P39" s="2"/>
+      <c r="Q39" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="R39" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="S39" s="2"/>
+    </row>
+    <row r="40" spans="1:19">
+      <c r="A40" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K40" s="2"/>
+      <c r="L40" s="2"/>
+      <c r="M40" s="2"/>
+      <c r="N40" s="2"/>
+      <c r="O40" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="P40" s="2"/>
+      <c r="Q40" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="R40" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="S40" s="2"/>
+    </row>
+    <row r="41" spans="1:19">
+      <c r="A41" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K41" s="2"/>
+      <c r="L41" s="2"/>
+      <c r="M41" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="N41" s="2"/>
+      <c r="O41" s="2"/>
+      <c r="P41" s="2"/>
+      <c r="Q41" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="R41" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="S41" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>